<commit_message>
Regenerate the published guide from the current sources
Runs the IG publisher over the sources changed in this lot, so the
published copy under site/public/ig matches them: the risk assessment
example now carries the point total in the heartland-risk-score-total
extension instead of probabilityDecimal, the blood pressure thresholds
that existed only in this guide are gone, and the new score extension
and code system have pages of their own.

Built with the terminology server switched off, because tx.fhir.org is
not reachable from this machine. That leaves one validation error and
several warnings that all say the same thing, that codes could not be
checked without a terminology service, and it drops qa-tx.html, which
only exists when a terminology server was used.

The disclaimer on the home page still says clinical decision support:
its source, input/pagecontent/index.md, has uncommitted edits belonging
to another change and was left alone.
</commit_message>
<xml_diff>
--- a/site/public/ig/StructureDefinition-heartland-remote-monitoring-observation.xlsx
+++ b/site/public/ig/StructureDefinition-heartland-remote-monitoring-observation.xlsx
@@ -63,7 +63,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-04-16T20:13:50-04:00</t>
+    <t>2026-09-17T14:02:25-04:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -90,7 +90,7 @@
     <t>Description</t>
   </si>
   <si>
-    <t>Observation captured via the HEARTLAND remote monitoring kit (Module 5): body weight, blood pressure (systolic/diastolic), or oxygen saturation. Red-flag thresholds are encoded via Observation.referenceRange with meaning.text identifying the rule. Default thresholds (HEARTLAND v3.2 standard, configurable per program): weight gain &gt;=2 lb (0.9 kg)/24h or &gt;=5 lb (2.3 kg)/7d; SBP &lt;90 or &gt;180 mmHg; DBP &lt;50 or &gt;110 mmHg; SpO2 &lt;90% on room air. Per the human filter principle, all non-emergency alerts pass through licensed clinician telephone assessment before ED referral.</t>
+    <t>Observation captured via the HEARTLAND remote monitoring kit (Module 5): body weight, blood pressure (systolic/diastolic), or oxygen saturation. Red-flag thresholds are encoded via Observation.referenceRange with meaning.text identifying the rule. The weight and oxygen saturation values a program configures here are starting defaults, not HEARTLAND Protocol rules: weight gain &gt;=2 lb (0.9 kg)/24h or &gt;=5 lb (2.3 kg)/7d, and SpO2 &lt;90% on room air, all configurable per program. Systolic BP &lt;90 mmHg is the only blood pressure red flag; this guide states no diastolic threshold and no high systolic threshold. Per the human filter principle, all non-emergency alerts pass through licensed clinician telephone assessment before ED referral.</t>
   </si>
   <si>
     <t>Purpose</t>

</xml_diff>